<commit_message>
Finishin Task Text Feature
</commit_message>
<xml_diff>
--- a/Task N-grams/abstract.xlsx
+++ b/Task N-grams/abstract.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2d3c97bd3821a9d6/Dokumen/Kuylah/SEM 2/RFPP/RFPP_Task/Task N-grams/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ammar\OneDrive\Dokumen\Kuylah\SEM 2\RFPP\RFPP_Task\Task N-grams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E37BEA3D-FAFA-4924-983F-13D3C4C8A541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540E0280-46C9-4CF7-B4EB-7E5A281165B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1170" yWindow="1170" windowWidth="14190" windowHeight="10350" xr2:uid="{A1C0CD0A-4EC4-4631-8455-5525592C40D0}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>title</t>
   </si>
@@ -42,9 +42,6 @@
     <t>abstrak_eng</t>
   </si>
   <si>
-    <t>In  the  digital  era,  sentiment  analysis has  become  crucial  to  evaluate  public  opinion, especially in the context of Play Storeapps with Indonesian-language reviews. This research aims to  improve  the  performance  of  the  IndoBERT  model  in  sentiment  analysis  of  DeepSeek  app reviews by using data augmentation and hyperparameter tuning techniques. Data augmentation is  done  through the back-translation  technique,  while  the  hyperparameters  tested  include  the number of epochs, learning rate, and batch size. Experimental results show that the combination of data augmentation with epoch 10, learning rate 2e-5, and batch size 16 produces thehighest accuracy  of  93.95%  and  F1-score  of  0.94,  with  better  stability  than  the  model  without augmentation. The model without augmentation showed fluctuations in performance, indicating overfitting   in   some   configurations.   These   findings   confirm   the   importance   of   applying augmentation techniques and hyperparameter tuning in improving the accuracy and stability of sentiment analysis models, and contribute to the development of NLP models for Indonesian and other resource-constrained languages</t>
-  </si>
-  <si>
     <t>abstrak_idn</t>
   </si>
   <si>
@@ -69,15 +66,28 @@
     <t>Developments and Trends in Indonesian Tourism Technology Using Bibliometric Analysis</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Personality classification using textual data from social media or online forums is a complex task due to the unstructured text and the multifaceted nature of personality. While the Myers-Briggs Type Indicator (MBTI) provides a comprehensive framework, adapting it to media data and handling diverse linguistic patterns requires effective algorithms. The psychological basis of MBTI is intricate, especially when using complex methods like deep learning, which can be challenging. 
-     This study classifies personality types based on each individual's behavior on an online forum by observing the linguistic patterns of posted textual data using the SVM, Random Forest, BERT, and Word2Vec algorithms. The SVM and Random Forest algorithms are traditional machine learning algorithms known for their capabilities and effectiveness in text classification. Meanwhile, BERT and Word2Vec identify semantic relationships and contextual information from textual data. In addition, the IndoBERT model will be used for the BERT model because this study focuses on the classification of Indonesian language texts.
-Testing was carried out using textual data from posts on the PersonalityCafe forum. The test results showed that the combination of the SVM and IndoBERT models outperformed other models with an accuracy rate of 82% and an F1 score of 75%.</t>
-  </si>
-  <si>
     <t>Personality Classification of Myers Briggs Type Indicators (MBTI) Using BERT and Machine Learning</t>
+  </si>
+  <si>
+    <t>Personality classification using textual data from social media or online forums is a complex task  due  to  the  unstructured  text  and  the  multifaceted  nature  of  personality.  While  the  Myers-Briggs Type Indicator (MBTI) provides a comprehensive framework, adapting it to media data and handling diverse linguistic patterns requires effective  algorithms. The psychological basis of MBTI is intricate, especially when using complex methods like deep learning, which can be challenging. This  study  classifies  personality  types  based  on  each  individual's  behavioron  an  online forum  by  observing  the  linguistic  patterns  of  posted  textual  data  using  the  SVM,  Random Forest,  BERT,  and  Word2Vec  algorithms.  The  SVM  and  Random  Forest  algorithms  are traditional  machine  learning  algorithms  known  for  their  capabilities  and  effectiveness  in  text classification. Meanwhile, BERT and Word2Vec identify semantic relationships and contextual information  from  textual  data.  In  addition,  the  IndoBERT  model  will  be  used  for  the  BERT model because this study focuses on the classification of Indonesian language texts.Testing was carried out using textual data from posts on the PersonalityCafe forum. The test results  showed  that  the  combination  of  the  SVM  and  IndoBERT  models  outperformed  other models with an accuracy rate of 82% and an F1 score of 75%</t>
+  </si>
+  <si>
+    <t>Klasifikasi  kepribadian  menggunakan  data  tekstual  yang  bersumber  dari  media  sosial ataupun  forum  daring  menimbulkan  berbagai  tantangan  yang  disebabkan  oleh  sifat  teks  yang tidak terstruktur dan kompleksitas penilaian kepribadian.Walaupun, model kepribadianMyers-Briggs    Type    Indicator (MBTI)    menyediakan    kerangka    kerja    yang    komprehensif, mengadaptasinya  ke  data  media  dan  menangani  pola linguistik  yang  beragammemerlukan algoritmayang  efektif. Selain  itu,  dasar  psikologismodelMBTI yang rumitdiklasifikasi, terutama saat menggunakan metode yang kompleksseperti pembelajaran mendalam.Penelitian  ini  mengklasifikasikan  tipe  kepribadian  berdasarkan  perilaku  masing-masing individu  pada  forum  online  dengan  memerhatikan  pola  linguistik  dari  data  tekstual  yang diunggah  menggunakan  algoritmaSVM,  Random  Forest,  BERT,  dan  Word2Vec.  Algoritma SVM  dan  Random  Forest  merupakan  algoritma  pembelajaran  mesin  tradisional  yang  dikenal dengan  kemampuan  dan  efektivitasnya  dalam  peran  klasifikasi  teks.  Sedangkan,  BERT  dan Word2Vec digunakan untuk mengidentifikasi hubungan semantik dan informasi kontekstual dari data tekstual. Selain itu, untuk model BERT akan digunakan model IndoBERT karena penelitian ini berfokus pada klasifikasi teks berbahasa Indonesia.Pengujian dilakukan dengan menggunakan data tekstual dari unggahan yang terdapatpada forum  PersonalityCafe.  Hasil  pengujian  menunjukkan  bahwa  kombinasi  model  SVM  dan IndoBERT  mengungguli model  lainnyadengan  tingkat  akurasi  sebesar  82%  dan  skor  F1sebesar 75%</t>
+  </si>
+  <si>
+    <t>Teknologi informasi telah mengubah masyarakat, layanan, juga sektor pariwisata telah menarik banyak penelitian dan publikasi. Meskipun penelitian terdahulu bertujuan menunjukkan pemahaman faktor teknologi pariwisata, tetapi masih kurang yang membahas faktor teknologi pariwisata  Indonesia.  Membahas  publikasi  ilmiah  tentang  teknologi  pariwisata  di  Indonesia dapat memberikan pemahaman lebih dalam tentang pengembangan teknologi informasi dalam sektor  pariwisata  Indonesia  dengan  memberikan  solusi.  penelitian  inibertujuan  menganalisis perkembangan dan tren faktor teknologi pariwisata di Indonesia dari tahun 2014 hingga 2023 dengan  analisis  bibliometric  dari  R  studio  serta  menggunakan  113  artikel  terindeks  scopus. Metodologi meliputi perencanaan, identifikasi katakunci, pencarian data scopus, bibliometric, perkembangan,  dan  tren  teknologi  pariwisata  Indonesia.  Hasil  penelitian  ini  didapatkan peningkatan  publikasi  dari  tahun  ke  tahun,  pada  kutipan  pertahun  terjadi  fluktuasi,Jumlah  artikel terpublikasi bervariasi dengan Sustainability (switzerland) menjadi peringkat pertama,, indonesia berkolaborasi dengan Malaysia, United Kingdom,Belgium, Indonesia juga menjadi top keywords serta tren topik, dan pada tren teknologi pariwisata terdapat dua klaster yang berada di   dalam   tematik   basic   themes   yaitu   tourism   dan   west   java   yang   menjadi   arah  untuk penelitianselanjutnya</t>
+  </si>
+  <si>
+    <t>Transfer Learning of Pre-trained Transformers forCovid-19 Hoax Detectionin Indonesian Language</t>
+  </si>
+  <si>
+    <t>Nowadays, internet has become the most popular source of news. However, the validity of the online news articles is difficult to assess, whether it is a fact or a hoax. Hoaxes relatedto Covid-19brought  a  problematic  effect to  human  life.  An  accurate  hoax  detection  system  is important  to  filter  abundant  information  on  the  internet.    In  this  research,a Covid-19  hoax detectionsystemwasproposed  by transfer  learning  of  pre-trainedtransformer models. Fine-tuned  original  pre-trained  BERT,  multilingual  pre-trained  mBERT,  and  monolingual  pre-trained IndoBERTwere usedto solve the classification taskin the hoax detection system. Based on  the  experimental  results, fine-tuned  IndoBERT models  trained  on  monolingual  Indonesian corpus outperform fine-tuned original and multilingual BERT with uncased versions. However, the fine-tuned mBERT cased model trainedona larger corpus achieved the best performance.</t>
+  </si>
+  <si>
+    <t>Pada saat ini, internet menjadi sumber berita paling populer. Akan tetapi, validitas dari artikel berita online sulit dinilai, apakah artikel tersebut berupa fakta atau hoaks. Hoaks terkait Covid-19  membawa  efek  problematik  terhadap  kehidupan  manusia.  Sistem  pendeteksi  hoaks yang  akurat  menjadi  penting  untuk  menyaring  informasi  yang  tersebar  di  internet. Pada penelitian  ini, sistem  pendeteksi  hoaks  diusulkan  dengan  menerapkan  transfer  learning  dari pre-trained transformer model. Fine-tuned original pre-trained BERT, multilingual pre-trained mBERT, danmonolingual   pre-trained   IndoBERTdigunakan   untuk   menyelesaikan   tugas klasifikasi pada  sistem pendeteksi  hoaks.Berdasarkan  hasil  eksperimen,modelfine-tuned IndoBERTyang  dilatih  di  korpusmonolingual berbahasa  Indonesialebih  baik  akurasinya dibandingkanfine-tuned  original danmultilingual  BERT dengan  versiuncased. Akan  tetapi, fine-tuned model mBERTdengan versicased yang dilatih di corpus yang lebih besar mencapai kinerja yang paling baik dibandingkan denganmodel lainnya.</t>
+  </si>
+  <si>
+    <t>In  the  digital  era,  sentiment  analysis has  become  crucial  to  evaluate  public  opinion, especially in the context of Play Storeapps with Indonesian-language reviews. This research aims to  improve  the  performance  of  the  IndoBERT  model  in  sentiment  analysis  of  DeepSeek  app reviews by using data augmentation and hyperparameter tuning techniques. Data augmentation is  done  through the back-translation  technique,  while  the  hyperparameters  tested  include  the number of epochs, learning rate, and batch size. Experimental results show that the combination of data augmentation with epoch 10, learning rate 2e-5, and batch size 16 produces thehighest accuracy  of  93.95%  and  F1-score  of  0.94,  with  better  stability  than  the  model  without augmentation. The model without augmentation showed fluctuations in performance, indicating overfitting   in   some   configurations.   These   findings   confirm   the   importance   of   applying augmentation techniques and hyperparameter tuning in improving the accuracy and stability of sentiment analysis models, and contribute to the development of NLP models for Indonesian and other resource-constrained languages.</t>
   </si>
 </sst>
 </file>
@@ -432,9 +442,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6B81842-9BBA-4E67-B978-F461068DF1DE}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="77" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -446,48 +457,62 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>